<commit_message>
Both накладная templates: install latest revisions
Both files changed again: the price накладная now has an explicit НДС
column (previously implied — Кол-во and Сумма без НДС also swapped order),
and its total row folds 'Итого:'+amount into one cell instead of a separate
'всего к оплате' label. The weekly накладная's Номер заказа/Сумма без ндс/
НДС columns went back to being 2-wide merges.

Generalized further while at it: downloadOrderExcelWithPrice now also reads
its totals-row label text off the template (like the weekly variant already
did) instead of assuming 'всего к оплате', and both exports share one
writeTemplateRow/writeTotalRow pair rather than keeping separate per-variant
copies — this is the third revision each template has been through this
week, and the column layout keeps moving, so less hand-transcribed text and
less duplicated row-writing logic means less to get wrong on the fourth.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/assets/templates/order-invoice-with-price-template.xlsx
+++ b/src/assets/templates/order-invoice-with-price-template.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>№</t>
   </si>
@@ -75,19 +75,22 @@
     <t>Сумма</t>
   </si>
   <si>
-    <t>всего к оплате</t>
-  </si>
-  <si>
     <t>[vat_amunt]</t>
   </si>
   <si>
-    <t>[total_amunt]</t>
-  </si>
-  <si>
     <t>Сумма без НДС</t>
   </si>
   <si>
     <t>[sum_without_vat]</t>
+  </si>
+  <si>
+    <t>НДС</t>
+  </si>
+  <si>
+    <t>[vat_sum]</t>
+  </si>
+  <si>
+    <t>Итого:[total_amunt]</t>
   </si>
 </sst>
 </file>
@@ -132,10 +135,12 @@
     </font>
     <font>
       <b/>
-      <sz val="8"/>
+      <sz val="11"/>
       <color indexed="8"/>
-      <name val="sans-serif"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <charset val="204"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -157,7 +162,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -228,20 +233,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -267,41 +263,59 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -620,16 +634,16 @@
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
-  <dimension ref="A1:U12"/>
+  <dimension ref="A1:V12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.140625" customWidth="1"/>
     <col min="2" max="2" width="34.28515625" customWidth="1"/>
-    <col min="3" max="4" width="18.140625" customWidth="1"/>
-    <col min="5" max="5" width="11.42578125" customWidth="1"/>
+    <col min="3" max="5" width="18.140625" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21">
+    <row r="1" spans="1:22">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -637,86 +651,94 @@
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
-    </row>
-    <row r="2" spans="1:21">
-      <c r="A2" s="21" t="s">
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" spans="1:22">
+      <c r="A2" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="21"/>
+      <c r="B2" s="15"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
-    </row>
-    <row r="3" spans="1:21">
-      <c r="A3" s="21" t="s">
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="1:22">
+      <c r="A3" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="21"/>
+      <c r="B3" s="28"/>
       <c r="C3" s="2"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="1"/>
-    </row>
-    <row r="4" spans="1:21" ht="15" customHeight="1">
-      <c r="A4" s="13" t="s">
+      <c r="D3" s="13"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="1"/>
+    </row>
+    <row r="4" spans="1:22" ht="15" customHeight="1">
+      <c r="A4" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="13"/>
+      <c r="B4" s="16"/>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
-    </row>
-    <row r="5" spans="1:21">
-      <c r="A5" s="13" t="s">
+      <c r="F4" s="4"/>
+    </row>
+    <row r="5" spans="1:22">
+      <c r="A5" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="13"/>
+      <c r="B5" s="16"/>
       <c r="C5" s="3"/>
       <c r="D5" s="4"/>
-      <c r="E5" s="3"/>
-      <c r="H5" s="1"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
-    </row>
-    <row r="6" spans="1:21">
-      <c r="A6" s="13" t="s">
+      <c r="M5" s="1"/>
+    </row>
+    <row r="6" spans="1:22">
+      <c r="A6" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="13"/>
+      <c r="B6" s="16"/>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
-      <c r="H6" s="9"/>
+      <c r="F6" s="4"/>
       <c r="I6" s="9"/>
-      <c r="J6" s="5"/>
+      <c r="J6" s="9"/>
       <c r="K6" s="5"/>
-      <c r="L6" s="1"/>
-    </row>
-    <row r="7" spans="1:21" ht="15" customHeight="1">
-      <c r="A7" s="13" t="s">
+      <c r="L6" s="5"/>
+      <c r="M6" s="1"/>
+    </row>
+    <row r="7" spans="1:22" ht="15" customHeight="1">
+      <c r="A7" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="13"/>
+      <c r="B7" s="16"/>
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
-      <c r="J7" s="13"/>
-      <c r="K7" s="13"/>
-      <c r="L7" s="13"/>
-    </row>
-    <row r="8" spans="1:21" ht="15" customHeight="1" thickBot="1">
-      <c r="A8" s="13" t="s">
+      <c r="F7" s="4"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="16"/>
+      <c r="L7" s="16"/>
+      <c r="M7" s="16"/>
+    </row>
+    <row r="8" spans="1:22" ht="15" customHeight="1" thickBot="1">
+      <c r="A8" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="13"/>
+      <c r="B8" s="16"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
-    </row>
-    <row r="9" spans="1:21" ht="15.75" thickBot="1">
+      <c r="F8" s="4"/>
+    </row>
+    <row r="9" spans="1:22" ht="15.75" thickBot="1">
       <c r="A9" s="6" t="s">
         <v>0</v>
       </c>
@@ -727,37 +749,42 @@
         <v>16</v>
       </c>
       <c r="D9" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="F9" s="15" t="s">
+      <c r="G9" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="G9" s="16"/>
-    </row>
-    <row r="10" spans="1:21" ht="34.5" thickBot="1">
+      <c r="H9" s="18"/>
+    </row>
+    <row r="10" spans="1:22" ht="34.5" thickBot="1">
       <c r="A10" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="D10" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F10" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="E10" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F10" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="G10" s="18"/>
-      <c r="H10" s="10"/>
+      <c r="G10" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="H10" s="26"/>
       <c r="I10" s="10"/>
       <c r="J10" s="10"/>
       <c r="K10" s="10"/>
@@ -771,25 +798,45 @@
       <c r="S10" s="10"/>
       <c r="T10" s="10"/>
       <c r="U10" s="10"/>
-    </row>
-    <row r="11" spans="1:21" ht="23.25" customHeight="1" thickBot="1">
-      <c r="A11" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="14"/>
-      <c r="F11" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="G11" s="20"/>
-      <c r="H11" s="1"/>
-    </row>
-    <row r="12" spans="1:21">
+      <c r="V10" s="10"/>
+    </row>
+    <row r="11" spans="1:22" ht="15.75" thickBot="1">
+      <c r="A11" s="21"/>
+      <c r="B11" s="22"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="H11" s="20"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="10"/>
+      <c r="O11" s="10"/>
+      <c r="P11" s="10"/>
+      <c r="Q11" s="10"/>
+      <c r="R11" s="10"/>
+      <c r="S11" s="10"/>
+      <c r="T11" s="10"/>
+      <c r="U11" s="10"/>
+      <c r="V11" s="10"/>
+    </row>
+    <row r="12" spans="1:22">
       <c r="A12" t="s">
         <v>9</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="11">
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="I7:M7"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="G10:H10"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A7:B7"/>
@@ -797,13 +844,8 @@
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A6:B6"/>
-    <mergeCell ref="H7:L7"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="F11:G11"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>